<commit_message>
changed the Search type in controller
</commit_message>
<xml_diff>
--- a/AML.Core.Web.API/AML.Web/Files/Data-Corporate Bulk upload Sample.xlsx
+++ b/AML.Core.Web.API/AML.Web/Files/Data-Corporate Bulk upload Sample.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GiteaProject\LemonWatchdog_03022026\lemon\AML.Core.Web.API\AML.Web\Files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GiteaProject\LemonUAT_05032026\lemon\AML.Core.Web.API\AML.Web\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0664A30F-D803-438C-A1CF-9B3881703BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2B6F7FA-E210-4164-890B-1B1379207945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="3396" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8964" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,12 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
-    <t>Customer ID (Mandatory field)</t>
-  </si>
-  <si>
-    <t>Full Name of the Entity</t>
-  </si>
-  <si>
     <t>Date of Incorporation</t>
   </si>
   <si>
@@ -52,6 +46,12 @@
   </si>
   <si>
     <t>Country of Incorporation</t>
+  </si>
+  <si>
+    <t>Customer ID</t>
+  </si>
+  <si>
+    <t>Full Name of the Entity(Mandatory)</t>
   </si>
 </sst>
 </file>
@@ -166,7 +166,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -509,31 +509,31 @@
   <sheetData>
     <row r="1" spans="1:9" ht="61.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="G1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">

</xml_diff>